<commit_message>
Incorporating location into the planning
</commit_message>
<xml_diff>
--- a/Documentation/GoapPlanningExample.xlsx
+++ b/Documentation/GoapPlanningExample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Morten Lang\source\repos\VirtualVillage\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65959A7E-7B24-4561-AAE3-15DF8A416445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C185549-89C8-439F-947C-E2FA3B12BA91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5535" yWindow="2175" windowWidth="25020" windowHeight="18585" xr2:uid="{8C3796D5-A4C5-4AE7-83D8-F5BFD42AC240}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="26415" windowHeight="14130" xr2:uid="{8C3796D5-A4C5-4AE7-83D8-F5BFD42AC240}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="68">
   <si>
     <t>Action</t>
   </si>
@@ -231,6 +231,15 @@
   </si>
   <si>
     <t>Plan</t>
+  </si>
+  <si>
+    <t>Wander</t>
+  </si>
+  <si>
+    <t>AtTarget[Random]</t>
+  </si>
+  <si>
+    <t>AtTarget[StoreHouse]</t>
   </si>
 </sst>
 </file>
@@ -635,7 +644,7 @@
     <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.140625" customWidth="1"/>
     <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17" customWidth="1"/>
+    <col min="14" max="14" width="21.5703125" customWidth="1"/>
     <col min="15" max="15" width="15.5703125" customWidth="1"/>
     <col min="16" max="16" width="11.42578125" customWidth="1"/>
     <col min="24" max="24" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -646,7 +655,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
         <v>12</v>
@@ -758,10 +767,10 @@
         <v>28</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
@@ -817,7 +826,7 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="E9" t="s">
         <v>53</v>

</xml_diff>